<commit_message>
Druhý pokrok - dodělat linky_otevreni cele nemam skoro vubec nic a zakomentovat vsechny radky popsat co delaji zacit delat dokumentaci
</commit_message>
<xml_diff>
--- a/zaverecny_projekt.xlsx
+++ b/zaverecny_projekt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\prokop_stepan\IdeaProjects\zaverecny_projekt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9997F29F-5514-4EEA-B5B1-D7AAAD9D268B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99073A8F-5FD2-471D-8F7A-D6EB185E47CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -118,7 +118,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -137,12 +137,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -193,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -202,7 +196,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
@@ -534,7 +527,7 @@
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="7" t="s">
         <v>4</v>
       </c>
     </row>
@@ -542,7 +535,7 @@
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="7" t="s">
         <v>5</v>
       </c>
     </row>
@@ -550,7 +543,7 @@
       <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>6</v>
       </c>
     </row>
@@ -558,7 +551,7 @@
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="7" t="s">
         <v>7</v>
       </c>
     </row>
@@ -566,7 +559,7 @@
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="7" t="s">
         <v>8</v>
       </c>
     </row>
@@ -582,7 +575,7 @@
       <c r="A9" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="7" t="s">
         <v>10</v>
       </c>
     </row>
@@ -590,7 +583,7 @@
       <c r="A10" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="7" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Třetí pokrok - dodělat zobrazování linek a rozdělat přihlášení a nákup jízdenek
</commit_message>
<xml_diff>
--- a/zaverecny_projekt.xlsx
+++ b/zaverecny_projekt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\prokop_stepan\IdeaProjects\zaverecny_projekt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99073A8F-5FD2-471D-8F7A-D6EB185E47CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D57D7DDE-9737-4F4F-8039-8D2646156188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="26">
   <si>
     <t>Sekce</t>
   </si>
@@ -86,6 +86,18 @@
   </si>
   <si>
     <t>Obhajoba – váha 9</t>
+  </si>
+  <si>
+    <t>Přihlášení</t>
+  </si>
+  <si>
+    <t>admin = admin123</t>
+  </si>
+  <si>
+    <t>jnakol = tajneheslo123</t>
+  </si>
+  <si>
+    <t>pavelknotek = jagercigo</t>
   </si>
 </sst>
 </file>
@@ -187,7 +199,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -196,6 +208,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
@@ -498,11 +511,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="64" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -625,10 +639,10 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>18</v>
       </c>
@@ -636,7 +650,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>18</v>
       </c>
@@ -644,13 +658,29 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>18</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>21</v>
       </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>